<commit_message>
Dados por subprefeitura em relação as descrições de funções
</commit_message>
<xml_diff>
--- a/R Markdown/resultados/funcoes_orcamentarias_por_subprefeitura.xlsx
+++ b/R Markdown/resultados/funcoes_orcamentarias_por_subprefeitura.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cloudprodamazhotmail-my.sharepoint.com/personal/gabrielmachado_prefeitura_sp_gov_br/Documents/Área de Trabalho/IDRGP/IDRGP-2025/R Markdown/resultados/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_25D688E632A63B2398DCF9CF1608D773AE301B47" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DD9CD377-0CF3-40CF-B127-8AA1CF938331}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="11_25D688E63246BF4480DCE4CF1608D773AE301B47" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C3B63569-3F4E-4AD0-A80F-EB203CE95C9F}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Recuperada_Planilha1" sheetId="1" r:id="rId1"/>
+    <sheet name="AF - Aricanduva" sheetId="1" r:id="rId1"/>
     <sheet name="BT - Butantã" sheetId="2" r:id="rId2"/>
     <sheet name="CL - Campo Limpo" sheetId="3" r:id="rId3"/>
     <sheet name="CS - Capela do Socorro" sheetId="4" r:id="rId4"/>
-    <sheet name="Recuperada_Planilha2" sheetId="5" r:id="rId5"/>
+    <sheet name="CV - Casa Verde" sheetId="5" r:id="rId5"/>
     <sheet name="AD - Cidade Ademar" sheetId="6" r:id="rId6"/>
     <sheet name="CT - Cidade Tiradentes" sheetId="7" r:id="rId7"/>
     <sheet name="EM - Ermelino Matarazzo" sheetId="8" r:id="rId8"/>

</xml_diff>